<commit_message>
Create User Stories in Documentation
Created User Stories for Students and Teachers for initial goals for Project/System.
Made 7 User Stories for Students and 6 User Stories for Teachers.
</commit_message>
<xml_diff>
--- a/documentation/Product Backlog.xlsx
+++ b/documentation/Product Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrocker1\Desktop\DevOps\Project\DevOps-F26-Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9371551-CA42-4945-8BEC-E63316B3B1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C4E72F-F08B-4484-9A4C-7EB7ACBC1688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
   <si>
     <t>Priority</t>
   </si>
@@ -37,6 +37,87 @@
   </si>
   <si>
     <t>So that…</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Create a Class</t>
+  </si>
+  <si>
+    <t>See how my class grade changes.</t>
+  </si>
+  <si>
+    <t>Average all my Classes</t>
+  </si>
+  <si>
+    <t>Determine my overall GPA</t>
+  </si>
+  <si>
+    <t>I can fix misinputs or add additional points.</t>
+  </si>
+  <si>
+    <t>Allow (x) Grades to be dropped</t>
+  </si>
+  <si>
+    <t>I can determine which grades are automatically dropped.</t>
+  </si>
+  <si>
+    <t>Teacher</t>
+  </si>
+  <si>
+    <t>I can input grades for students.</t>
+  </si>
+  <si>
+    <t>Add a Student</t>
+  </si>
+  <si>
+    <t>Delete Grade(s)</t>
+  </si>
+  <si>
+    <t>Change Grade(s)</t>
+  </si>
+  <si>
+    <t>Input Grade(s)</t>
+  </si>
+  <si>
+    <t>I can start inputting grades for them.</t>
+  </si>
+  <si>
+    <t>Remove a Student</t>
+  </si>
+  <si>
+    <t>I can remove them from my list if they drop the class.</t>
+  </si>
+  <si>
+    <t>Create an Assignment</t>
+  </si>
+  <si>
+    <t>I can input grades for all of my students.</t>
+  </si>
+  <si>
+    <t>Remove an Assignment</t>
+  </si>
+  <si>
+    <t>I can remove an assignment that will not count for a grade.</t>
+  </si>
+  <si>
+    <t>Input Grade for a Student</t>
+  </si>
+  <si>
+    <t>I can keep track of grades in my class.</t>
+  </si>
+  <si>
+    <t>I can input grades into a class.</t>
+  </si>
+  <si>
+    <t>I can remove grades that do not count towards my class.</t>
+  </si>
+  <si>
+    <t>Create SubSections</t>
+  </si>
+  <si>
+    <t>I can properly set weights on assignments towards overall class grade.</t>
   </si>
 </sst>
 </file>
@@ -78,9 +159,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,10 +451,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="4" width="30.6328125" customWidth="1"/>
+    <col min="3" max="3" width="30.6328125" customWidth="1"/>
+    <col min="4" max="4" width="59.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -381,6 +472,242 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>2</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>2</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>2</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>2</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="2"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Created New Project File
Created course_grade_calculator project.
Added modules similar to sample.
Added Ignore for module-info in devops_checks, it is a known issue from checkstyle and solution came from them.
Created Grade Class, tested all methods and got 100% code coverage.
Updated gitignore to ignore the target file.
</commit_message>
<xml_diff>
--- a/documentation/Product Backlog.xlsx
+++ b/documentation/Product Backlog.xlsx
@@ -8,24 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrocker1\Desktop\DevOps\Project\DevOps-F26-Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C4E72F-F08B-4484-9A4C-7EB7ACBC1688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF3243C0-0926-44A7-9ACD-6F6FC8849382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="0" windowWidth="25580" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>Priority</t>
   </si>
@@ -118,6 +127,12 @@
   </si>
   <si>
     <t>I can properly set weights on assignments towards overall class grade.</t>
+  </si>
+  <si>
+    <t>Use a pre-built Rubric</t>
+  </si>
+  <si>
+    <t>I can easily create a class instead of making all subsections</t>
   </si>
 </sst>
 </file>
@@ -575,13 +590,13 @@
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -592,10 +607,10 @@
         <v>12</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -606,10 +621,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -620,10 +635,10 @@
         <v>12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -634,10 +649,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -648,17 +663,25 @@
         <v>12</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>2</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>

</xml_diff>